<commit_message>
Workpaper 13_1: remove Y/Y/Y result codes, add annual-execution note to attribute 4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TL6bHHvGD5mcHDaTAY6zMH
</commit_message>
<xml_diff>
--- a/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_13_1.xlsx
+++ b/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_13_1.xlsx
@@ -1352,11 +1352,17 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>BSI.IT.6.C7.3</author>
+    <author>Control Testing</author>
   </authors>
   <commentList>
     <comment ref="B4" authorId="0" shapeId="0">
       <text>
         <t>Click an evidence file path to open the file. The evidence folder location is set on tab 'WP Summary' (yellow cell, row 27): blank = folder 'BSI.IT.6.C7.3-Evidences' next to this workbook.</t>
+      </text>
+    </comment>
+    <comment ref="A15" authorId="1" shapeId="0">
+      <text>
+        <t>Annual execution: 2025 cycle, BSI IT DR Exercise 11/15/2025 (DIV validated 11/15/2025), within the review period 08/01/2025 to 06/01/2026. 2024 cycle, Full DR Test (Virginia) 10/19/2024, see tab 'DR 2024 Testing Results'. One DR / DIV exercise per annual cycle; 392 days between exercises.</t>
       </text>
     </comment>
   </commentList>
@@ -1367,11 +1373,17 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>BSI.IT.6.C7.3</author>
+    <author>Control Testing</author>
   </authors>
   <commentList>
     <comment ref="B4" authorId="0" shapeId="0">
       <text>
         <t>Click an evidence file path to open the file. The evidence folder location is set on tab 'WP Summary' (yellow cell, row 27): blank = folder 'BSI.IT.6.C7.3-Evidences' next to this workbook.</t>
+      </text>
+    </comment>
+    <comment ref="A15" authorId="1" shapeId="0">
+      <text>
+        <t>Annual execution: 2025 cycle, BSI IT DR Exercise 11/15/2025 (DIV validated 11/15/2025), within the review period 08/01/2025 to 06/01/2026. 2024 cycle, Full DR Test (Virginia) 10/19/2024, see tab 'DR 2024 Testing Results'. One DR / DIV exercise per annual cycle; 392 days between exercises.</t>
       </text>
     </comment>
   </commentList>
@@ -5256,7 +5268,7 @@
       </c>
       <c r="S3" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
         </is>
       </c>
     </row>
@@ -5292,7 +5304,7 @@
       </c>
       <c r="G4" s="42" t="inlineStr">
         <is>
-          <t>11/15/2025, data validated during the DR exercise; Format / Headers / Content = Y / Y / Y for 1 of 1 record; no data integrity exceptions.</t>
+          <t>11/15/2025, data validated during the DR exercise; Format, Headers and Content validated for 1 of 1 record; no data integrity exceptions.</t>
         </is>
       </c>
       <c r="H4" s="42" t="inlineStr">
@@ -5368,7 +5380,7 @@
       </c>
       <c r="S4" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
         </is>
       </c>
     </row>
@@ -5404,7 +5416,7 @@
       </c>
       <c r="G5" s="42" t="inlineStr">
         <is>
-          <t>11/15/2025, data validated during the DR exercise; Format / Headers / Content = Y / Y / Y for 1 of 1 record; no data integrity exceptions.</t>
+          <t>11/15/2025, data validated during the DR exercise; Format, Headers and Content validated for 1 of 1 record; no data integrity exceptions.</t>
         </is>
       </c>
       <c r="H5" s="42" t="inlineStr">
@@ -5480,7 +5492,7 @@
       </c>
       <c r="S5" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
         </is>
       </c>
     </row>
@@ -5521,7 +5533,7 @@
       </c>
       <c r="G6" s="42" t="inlineStr">
         <is>
-          <t>11/15/2025, data validated during the DR exercise; Format / Headers / Content = Y / Y / Y for 6 of 6 records; no data integrity exceptions.</t>
+          <t>11/15/2025, data validated during the DR exercise; Format, Headers and Content validated for 6 of 6 records; no data integrity exceptions.</t>
         </is>
       </c>
       <c r="H6" s="42" t="inlineStr">
@@ -5614,7 +5626,7 @@
       </c>
       <c r="S6" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Claudia Romero, Miguel Orozco, Maria del Cerro Hontanilla).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Claudia Romero, Miguel Orozco, Maria del Cerro Hontanilla).</t>
         </is>
       </c>
     </row>
@@ -5650,7 +5662,7 @@
       </c>
       <c r="G7" s="42" t="inlineStr">
         <is>
-          <t>11/15/2025, data validated during the DR exercise; Format / Headers / Content = Y / Y / Y for 1 of 1 record; no data integrity exceptions.</t>
+          <t>11/15/2025, data validated during the DR exercise; Format, Headers and Content validated for 1 of 1 record; no data integrity exceptions.</t>
         </is>
       </c>
       <c r="H7" s="42" t="inlineStr">
@@ -5725,7 +5737,7 @@
       </c>
       <c r="S7" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Michelle Oropesa).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Michelle Oropesa).</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5773,7 @@
       </c>
       <c r="G8" s="42" t="inlineStr">
         <is>
-          <t>11/15/2025, data validated during the DR exercise; Format / Headers / Content = Y / Y / Y for 2 of 2 records; no data integrity exceptions.</t>
+          <t>11/15/2025, data validated during the DR exercise; Format, Headers and Content validated for 2 of 2 records; no data integrity exceptions.</t>
         </is>
       </c>
       <c r="H8" s="42" t="inlineStr">
@@ -5839,7 +5851,7 @@
       </c>
       <c r="S8" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Franklin Puentes).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Franklin Puentes).</t>
         </is>
       </c>
     </row>
@@ -5877,7 +5889,7 @@
       </c>
       <c r="G9" s="42" t="inlineStr">
         <is>
-          <t>11/15/2025, data validated during the DR exercise; Format / Headers / Content = Y / Y / Y for 5 of 5 records; no data integrity exceptions.</t>
+          <t>11/15/2025, data validated during the DR exercise; Format, Headers and Content validated for 5 of 5 records; no data integrity exceptions.</t>
         </is>
       </c>
       <c r="H9" s="42" t="inlineStr">
@@ -5966,7 +5978,7 @@
       </c>
       <c r="S9" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Franklin Puentes, Maria del Cerro Hontanilla).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Franklin Puentes, Maria del Cerro Hontanilla).</t>
         </is>
       </c>
     </row>
@@ -6002,7 +6014,7 @@
       </c>
       <c r="G10" s="42" t="inlineStr">
         <is>
-          <t>11/15/2025, data validated during the DR exercise; Format / Headers / Content = Y / Y / Y for 1 of 1 record; no data integrity exceptions.</t>
+          <t>11/15/2025, data validated during the DR exercise; Format, Headers and Content validated for 1 of 1 record; no data integrity exceptions.</t>
         </is>
       </c>
       <c r="H10" s="42" t="inlineStr">
@@ -6078,7 +6090,7 @@
       </c>
       <c r="S10" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Sadis Alvarenga Hernandez).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Sadis Alvarenga Hernandez).</t>
         </is>
       </c>
     </row>
@@ -6115,7 +6127,7 @@
       </c>
       <c r="G11" s="42" t="inlineStr">
         <is>
-          <t>11/15/2025, data validated during the DR exercise; Format / Headers / Content = Y / Y / Y for 2 of 2 records; no data integrity exceptions.</t>
+          <t>11/15/2025, data validated during the DR exercise; Format, Headers and Content validated for 2 of 2 records; no data integrity exceptions.</t>
         </is>
       </c>
       <c r="H11" s="45" t="inlineStr">
@@ -6197,7 +6209,7 @@
       </c>
       <c r="S11" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Michelle Oropesa).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Michelle Oropesa).</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6261,7 @@
       </c>
       <c r="G12" s="42" t="inlineStr">
         <is>
-          <t>11/15/2025, data validated during the DR exercise; Format / Headers / Content = Y / Y / Y for 36 of 36 records; no data integrity exceptions.</t>
+          <t>11/15/2025, data validated during the DR exercise; Format, Headers and Content validated for 36 of 36 records; no data integrity exceptions.</t>
         </is>
       </c>
       <c r="H12" s="42" t="inlineStr">
@@ -6386,7 +6398,7 @@
       </c>
       <c r="S12" s="44" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Ricardo Garcia, David Marquez, Claudia Romero, Miguel Orozco, Sadis Alvarenga Hernandez, Maria del Cerro Hontanilla, Michelle Oropesa, Franklin Puentes, Martha Sullivan, Liliana Vizhnay, Victoria Fernandez, Xavier Caisapanta, Clara De Castro).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Ricardo Garcia, David Marquez, Claudia Romero, Miguel Orozco, Sadis Alvarenga Hernandez, Maria del Cerro Hontanilla, Michelle Oropesa, Franklin Puentes, Martha Sullivan, Liliana Vizhnay, Victoria Fernandez, Xavier Caisapanta, Clara De Castro).</t>
         </is>
       </c>
     </row>
@@ -6967,7 +6979,7 @@
       </c>
       <c r="H16" s="67" t="n"/>
     </row>
-    <row r="17" ht="126" customHeight="1" s="50">
+    <row r="17" ht="190" customHeight="1" s="50">
       <c r="A17" s="78" t="inlineStr">
         <is>
           <t>E01</t>
@@ -7002,9 +7014,7 @@
 Checked for IT DR exercise name, was the exercise annually executed?
 Exercise Date 12/11/2025 / 2025 DR Test Scope = True
 Exercise Date 11/15/2025 / 2025 DR Test Scope = True
-2025 cycle: BSI IT DR Exercise 11/15/2025 (within the review period 08/01/2025 to 06/01/2026).
-2024 cycle: 2024 Full 2024 DR Test (Virginia) 10/19/2024, see tab 'DR 2024 Testing Results'.
-Interval 10/19/2024 to 11/15/2025 = 392 days; one DR / DIV exercise in each annual cycle.</t>
+Note: Annual execution: 2025 cycle, BSI IT DR Exercise 11/15/2025 (DIV validated 11/15/2025), within the review period 08/01/2025 to 06/01/2026. 2024 cycle, Full DR Test (Virginia) 10/19/2024, see tab 'DR 2024 Testing Results'. One DR / DIV exercise per annual cycle; 392 days between exercises.</t>
         </is>
       </c>
       <c r="F17" s="76" t="inlineStr">
@@ -7137,7 +7147,7 @@
       </c>
       <c r="E21" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Business Tester:
 'Business Tester(s)' column</t>
         </is>
@@ -7273,9 +7283,9 @@
       </c>
       <c r="E25" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Business Data validation:
-Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y</t>
+Business Data Validation Date 11/15/2025; Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="F25" s="76" t="inlineStr">
@@ -7410,7 +7420,7 @@
       </c>
       <c r="E29" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Business line manager name:
 'Department Manager' column</t>
         </is>
@@ -7553,7 +7563,7 @@
       </c>
       <c r="E33" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Business line manager approval dates:
 'Department Manager Approval Date' and 'Attestation Date' columns</t>
         </is>
@@ -7696,7 +7706,7 @@
       </c>
       <c r="E37" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for DIV Test procedures listed within the Test results document:
 'Data Integrity Validation Procedures' column</t>
         </is>
@@ -7919,7 +7929,7 @@
       </c>
       <c r="E43" s="76" t="inlineStr">
         <is>
-          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all Y/Y/Y; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.
+          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all validated; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.
 Checked for Emails showing Business line manager approval of DIV testing results:
 Application / record agreed to the evidence.</t>
         </is>
@@ -8126,9 +8136,9 @@
       </c>
       <c r="E49" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for All evidence of Data Integrity DR test in BCIC:
-BCiC DIV export (tester, dates, manager, Y/N results, attestation)</t>
+BCiC DIV export (tester, dates, manager, validation results, attestation)</t>
         </is>
       </c>
       <c r="F49" s="76" t="inlineStr">
@@ -8628,7 +8638,7 @@
       </c>
       <c r="E63" s="76" t="inlineStr">
         <is>
-          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all Y/Y/Y; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.
+          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all validated; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.
 Checked for Business Line Approval of Results:
 Application / record agreed to the evidence.</t>
         </is>
@@ -8835,7 +8845,7 @@
       </c>
       <c r="E69" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Results Documented in BCMS:
 DIV results, business tester, validation date, manager approval and attestation fields recorded in BCMS (BC in the Cloud) for each application</t>
         </is>
@@ -8938,7 +8948,7 @@
       </c>
       <c r="E73" s="76" t="inlineStr">
         <is>
-          <t>DR test script with Data Integrity Validation section. Application in-scope: FedImport, FedExport, Imaging101, T24. Format / Headers / Content = Y, "No data discrepancy found". Steps include ACH Express import and Imaging101 validation screenshots (14 pages).</t>
+          <t>DR test script with Data Integrity Validation section. Application in-scope: FedImport, FedExport, Imaging101, T24. Format, Headers and Content validated, "No data discrepancy found". Steps include ACH Express import and Imaging101 validation screenshots (14 pages).</t>
         </is>
       </c>
       <c r="F73" s="76" t="inlineStr">
@@ -9249,7 +9259,7 @@
       </c>
       <c r="E83" s="76" t="inlineStr">
         <is>
-          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all Y/Y/Y; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.</t>
+          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all validated; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.</t>
         </is>
       </c>
       <c r="F83" s="76" t="inlineStr">
@@ -9848,7 +9858,7 @@
       </c>
       <c r="E101" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
         </is>
       </c>
       <c r="F101" s="76" t="inlineStr">
@@ -9884,7 +9894,7 @@
       </c>
       <c r="E102" s="76" t="inlineStr">
         <is>
-          <t>BCiC 'Data Integrity Validation Testing' screen (1 to 20 of 66 items) showing tester, validation date, manager, approval date, Y/N results and attestation fields.</t>
+          <t>BCiC 'Data Integrity Validation Testing' screen (1 to 20 of 66 items) showing tester, validation date, manager, approval date, validation results and attestation fields.</t>
         </is>
       </c>
       <c r="F102" s="76" t="inlineStr">
@@ -10272,7 +10282,7 @@
       </c>
       <c r="F115" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
         </is>
       </c>
       <c r="G115" s="77" t="inlineStr">
@@ -10334,7 +10344,7 @@
       </c>
       <c r="F116" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
         </is>
       </c>
       <c r="G116" s="77" t="inlineStr">
@@ -10396,7 +10406,7 @@
       </c>
       <c r="F117" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
         </is>
       </c>
       <c r="G117" s="77" t="inlineStr">
@@ -10461,7 +10471,7 @@
       </c>
       <c r="F118" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Claudia Romero, Miguel Orozco, Maria del Cerro Hontanilla).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Claudia Romero, Miguel Orozco, Maria del Cerro Hontanilla).</t>
         </is>
       </c>
       <c r="G118" s="77" t="inlineStr">
@@ -10522,7 +10532,7 @@
       </c>
       <c r="F119" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Michelle Oropesa).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Michelle Oropesa).</t>
         </is>
       </c>
       <c r="G119" s="77" t="inlineStr">
@@ -10585,7 +10595,7 @@
       </c>
       <c r="F120" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Franklin Puentes).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Franklin Puentes).</t>
         </is>
       </c>
       <c r="G120" s="77" t="inlineStr">
@@ -10650,7 +10660,7 @@
       </c>
       <c r="F121" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Franklin Puentes, Maria del Cerro Hontanilla).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Franklin Puentes, Maria del Cerro Hontanilla).</t>
         </is>
       </c>
       <c r="G121" s="77" t="inlineStr">
@@ -10712,7 +10722,7 @@
       </c>
       <c r="F122" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Sadis Alvarenga Hernandez).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Sadis Alvarenga Hernandez).</t>
         </is>
       </c>
       <c r="G122" s="77" t="inlineStr">
@@ -10776,7 +10786,7 @@
       </c>
       <c r="F123" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Michelle Oropesa).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Michelle Oropesa).</t>
         </is>
       </c>
       <c r="G123" s="77" t="inlineStr">
@@ -10856,7 +10866,7 @@
       </c>
       <c r="F124" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Ricardo Garcia, David Marquez, Claudia Romero, Miguel Orozco, Sadis Alvarenga Hernandez, Maria del Cerro Hontanilla, Michelle Oropesa, Franklin Puentes, Martha Sullivan, Liliana Vizhnay, Victoria Fernandez, Xavier Caisapanta, Clara De Castro).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Ricardo Garcia, David Marquez, Claudia Romero, Miguel Orozco, Sadis Alvarenga Hernandez, Maria del Cerro Hontanilla, Michelle Oropesa, Franklin Puentes, Martha Sullivan, Liliana Vizhnay, Victoria Fernandez, Xavier Caisapanta, Clara De Castro).</t>
         </is>
       </c>
       <c r="G124" s="77" t="inlineStr">
@@ -11837,7 +11847,7 @@
       <c r="AX16" s="85" t="n"/>
       <c r="AY16" s="85" t="n"/>
     </row>
-    <row r="17" ht="126" customHeight="1" s="50">
+    <row r="17" ht="190" customHeight="1" s="50">
       <c r="A17" s="78" t="inlineStr">
         <is>
           <t>E01</t>
@@ -11872,9 +11882,7 @@
 Checked for IT DR exercise name, was the exercise annually executed?
 Exercise Date 12/11/2025 / 2025 DR Test Scope = True
 Exercise Date 11/15/2025 / 2025 DR Test Scope = True
-2025 cycle: BSI IT DR Exercise 11/15/2025 (within the review period 08/01/2025 to 06/01/2026).
-2024 cycle: 2024 Full 2024 DR Test (Virginia) 10/19/2024, see tab 'DR 2024 Testing Results'.
-Interval 10/19/2024 to 11/15/2025 = 392 days; one DR / DIV exercise in each annual cycle.</t>
+Note: Annual execution: 2025 cycle, BSI IT DR Exercise 11/15/2025 (DIV validated 11/15/2025), within the review period 08/01/2025 to 06/01/2026. 2024 cycle, Full DR Test (Virginia) 10/19/2024, see tab 'DR 2024 Testing Results'. One DR / DIV exercise per annual cycle; 392 days between exercises.</t>
         </is>
       </c>
       <c r="F17" s="76" t="inlineStr">
@@ -12103,7 +12111,7 @@
       </c>
       <c r="E21" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Business Tester:
 'Business Tester(s)' column</t>
         </is>
@@ -12335,9 +12343,9 @@
       </c>
       <c r="E25" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Business Data validation:
-Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y</t>
+Business Data Validation Date 11/15/2025; Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="F25" s="76" t="inlineStr">
@@ -12568,7 +12576,7 @@
       </c>
       <c r="E29" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Business line manager name:
 'Department Manager' column</t>
         </is>
@@ -12807,7 +12815,7 @@
       </c>
       <c r="E33" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Business line manager approval dates:
 'Department Manager Approval Date' and 'Attestation Date' columns</t>
         </is>
@@ -13046,7 +13054,7 @@
       </c>
       <c r="E37" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for DIV Test procedures listed within the Test results document:
 'Data Integrity Validation Procedures' column</t>
         </is>
@@ -13413,7 +13421,7 @@
       </c>
       <c r="E43" s="76" t="inlineStr">
         <is>
-          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all Y/Y/Y; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.
+          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all validated; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.
 Checked for Emails showing Business line manager approval of DIV testing results:
 Application / record agreed to the evidence.</t>
         </is>
@@ -13764,9 +13772,9 @@
       </c>
       <c r="E49" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for All evidence of Data Integrity DR test in BCIC:
-BCiC DIV export (tester, dates, manager, Y/N results, attestation)</t>
+BCiC DIV export (tester, dates, manager, validation results, attestation)</t>
         </is>
       </c>
       <c r="F49" s="76" t="inlineStr">
@@ -14602,7 +14610,7 @@
       </c>
       <c r="E63" s="76" t="inlineStr">
         <is>
-          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all Y/Y/Y; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.
+          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all validated; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.
 Checked for Business Line Approval of Results:
 Application / record agreed to the evidence.</t>
         </is>
@@ -14953,7 +14961,7 @@
       </c>
       <c r="E69" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.
 Checked for Results Documented in BCMS:
 DIV results, business tester, validation date, manager approval and attestation fields recorded in BCMS (BC in the Cloud) for each application</t>
         </is>
@@ -15152,7 +15160,7 @@
       </c>
       <c r="E73" s="76" t="inlineStr">
         <is>
-          <t>DR test script with Data Integrity Validation section. Application in-scope: FedImport, FedExport, Imaging101, T24. Format / Headers / Content = Y, "No data discrepancy found". Steps include ACH Express import and Imaging101 validation screenshots (14 pages).</t>
+          <t>DR test script with Data Integrity Validation section. Application in-scope: FedImport, FedExport, Imaging101, T24. Format, Headers and Content validated, "No data discrepancy found". Steps include ACH Express import and Imaging101 validation screenshots (14 pages).</t>
         </is>
       </c>
       <c r="F73" s="76" t="inlineStr">
@@ -15703,7 +15711,7 @@
       </c>
       <c r="E83" s="76" t="inlineStr">
         <is>
-          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all Y/Y/Y; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.</t>
+          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all validated; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.</t>
         </is>
       </c>
       <c r="F83" s="76" t="inlineStr">
@@ -16734,7 +16742,7 @@
       </c>
       <c r="E101" s="76" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
         </is>
       </c>
       <c r="F101" s="76" t="inlineStr">
@@ -16794,7 +16802,7 @@
       </c>
       <c r="E102" s="76" t="inlineStr">
         <is>
-          <t>BCiC 'Data Integrity Validation Testing' screen (1 to 20 of 66 items) showing tester, validation date, manager, approval date, Y/N results and attestation fields.</t>
+          <t>BCiC 'Data Integrity Validation Testing' screen (1 to 20 of 66 items) showing tester, validation date, manager, approval date, validation results and attestation fields.</t>
         </is>
       </c>
       <c r="F102" s="76" t="inlineStr">
@@ -17086,22 +17094,22 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A80:G80"/>
+    <mergeCell ref="A67:G67"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A55:G55"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A96:G96"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A67:G67"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A39:G39"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A7:G7"/>
     <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A71:G71"/>
     <mergeCell ref="A51:G51"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A80:G80"/>
-    <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A55:G55"/>
-    <mergeCell ref="A71:G71"/>
     <mergeCell ref="A47:G47"/>
     <mergeCell ref="A23:G23"/>
   </mergeCells>
@@ -17562,7 +17570,7 @@
       </c>
       <c r="F5" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero).</t>
         </is>
       </c>
       <c r="G5" s="77" t="inlineStr">
@@ -17670,7 +17678,7 @@
       </c>
       <c r="F6" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Claudia Romero, Miguel Orozco, Maria del Cerro Hontanilla).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Claudia Romero, Miguel Orozco, Maria del Cerro Hontanilla).</t>
         </is>
       </c>
       <c r="G6" s="77" t="inlineStr">
@@ -17774,7 +17782,7 @@
       </c>
       <c r="F7" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Michelle Oropesa).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Michelle Oropesa).</t>
         </is>
       </c>
       <c r="G7" s="77" t="inlineStr">
@@ -17880,7 +17888,7 @@
       </c>
       <c r="F8" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Franklin Puentes).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Franklin Puentes).</t>
         </is>
       </c>
       <c r="G8" s="77" t="inlineStr">
@@ -17988,7 +17996,7 @@
       </c>
       <c r="F9" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Franklin Puentes, Maria del Cerro Hontanilla).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Franklin Puentes, Maria del Cerro Hontanilla).</t>
         </is>
       </c>
       <c r="G9" s="77" t="inlineStr">
@@ -18093,7 +18101,7 @@
       </c>
       <c r="F10" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Sadis Alvarenga Hernandez).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Sadis Alvarenga Hernandez).</t>
         </is>
       </c>
       <c r="G10" s="77" t="inlineStr">
@@ -18200,7 +18208,7 @@
       </c>
       <c r="F11" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Michelle Oropesa).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Michelle Oropesa).</t>
         </is>
       </c>
       <c r="G11" s="77" t="inlineStr">
@@ -18323,7 +18331,7 @@
       </c>
       <c r="F12" s="76" t="inlineStr">
         <is>
-          <t>PASS. DIV executed and validated (Y/Y/Y) during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Ricardo Garcia, David Marquez, Claudia Romero, Miguel Orozco, Sadis Alvarenga Hernandez, Maria del Cerro Hontanilla, Michelle Oropesa, Franklin Puentes, Martha Sullivan, Liliana Vizhnay, Victoria Fernandez, Xavier Caisapanta, Clara De Castro).</t>
+          <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Ricardo Garcia, David Marquez, Claudia Romero, Miguel Orozco, Sadis Alvarenga Hernandez, Maria del Cerro Hontanilla, Michelle Oropesa, Franklin Puentes, Martha Sullivan, Liliana Vizhnay, Victoria Fernandez, Xavier Caisapanta, Clara De Castro).</t>
         </is>
       </c>
       <c r="G12" s="77" t="inlineStr">
@@ -21331,9 +21339,9 @@
       </c>
       <c r="E5" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 47, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 48 to 11/15/2025; Y / Y / Y
-BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format / Headers / Content = Y, "No data discrepancy found"); pp.2-14 screenshots</t>
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 47, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 48 to 11/15/2025; Format, Headers and Content validated
+BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format, Headers and Content validated, "No data discrepancy found"); pp.2-14 screenshots</t>
         </is>
       </c>
       <c r="F5" s="25" t="inlineStr">
@@ -21365,7 +21373,7 @@
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 47, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 47, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 48, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, BCiC report screen (record on a later page of the 66-item report)
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 3
@@ -21387,7 +21395,7 @@
 DMA02: BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg, attached signed attestation section 1-2, IT DR team facilitates DIV performed by business line testers during actual DR testing
 BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 E09: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg, IT DR (Elizabeth Noda) issued test script, collected evidence and requested approval
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 47, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 47, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">
@@ -21475,10 +21483,10 @@
       </c>
       <c r="E6" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 9, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 9 to 11/15/2025; Y / Y / Y
-E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and Y/N columns
-BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format / Headers / Content = Y, "No data discrepancy found"); pp.2-14 screenshots</t>
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 9, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 9 to 11/15/2025; Format, Headers and Content validated
+E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and validation result columns
+BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format, Headers and Content validated, "No data discrepancy found"); pp.2-14 screenshots</t>
         </is>
       </c>
       <c r="F6" s="25" t="inlineStr">
@@ -21512,7 +21520,7 @@
       </c>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 9, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 9, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 9, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, records visible on screen
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 19
@@ -21534,7 +21542,7 @@
 DMA02: BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg, attached signed attestation section 1-2, IT DR team facilitates DIV performed by business line testers during actual DR testing
 BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 E09: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg, IT DR (Elizabeth Noda) issued test script, collected evidence and requested approval
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 9, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 9, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M6" s="25" t="inlineStr">
@@ -21622,10 +21630,10 @@
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 10, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 10 to 11/15/2025; Y / Y / Y
-E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and Y/N columns
-BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format / Headers / Content = Y, "No data discrepancy found"); pp.2-14 screenshots</t>
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 10, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 10 to 11/15/2025; Format, Headers and Content validated
+E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and validation result columns
+BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format, Headers and Content validated, "No data discrepancy found"); pp.2-14 screenshots</t>
         </is>
       </c>
       <c r="F7" s="25" t="inlineStr">
@@ -21659,7 +21667,7 @@
       </c>
       <c r="J7" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 10, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 10, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 10, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, records visible on screen
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 20
@@ -21681,7 +21689,7 @@
 DMA02: BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg, attached signed attestation section 1-2, IT DR team facilitates DIV performed by business line testers during actual DR testing
 BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 E09: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg, IT DR (Elizabeth Noda) issued test script, collected evidence and requested approval
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 10, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 10, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M7" s="25" t="inlineStr">
@@ -21771,10 +21779,10 @@
       </c>
       <c r="E8" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 5, 11, 13, 51, 53, 57, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 5, 11, 13, 52, 54, 58 to 11/15/2025; Y / Y / Y
-E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and Y/N columns
-BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format / Headers / Content = Y, "No data discrepancy found"); pp.2-14 screenshots
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 5, 11, 13, 51, 53, 57, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 5, 11, 13, 52, 54, 58 to 11/15/2025; Format, Headers and Content validated
+E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and validation result columns
+BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format, Headers and Content validated, "No data discrepancy found"); pp.2-14 screenshots
 BLA02: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf, p.1 DIV procedure &amp; in-scope apps; pp.2-14 production-day 11/14 versus test-day 11/15 screenshots</t>
         </is>
       </c>
@@ -21819,7 +21827,7 @@
       </c>
       <c r="J8" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 5, 11, 13, 51, 53, 57, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 5, 11, 13, 51, 53, 57, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 5, 11, 13, 52, 54, 58, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, records visible on screen
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 24
@@ -21843,7 +21851,7 @@
 BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 BLA02: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 E09: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg, IT DR (Elizabeth Noda) issued test script, collected evidence and requested approval
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 5, 11, 13, 51, 53, 57, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 5, 11, 13, 51, 53, 57, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M8" s="25" t="inlineStr">
@@ -21936,8 +21944,8 @@
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 61, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 62 to 11/15/2025; Y / Y / Y
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 61, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 62 to 11/15/2025; Format, Headers and Content validated
 BLA04: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx, DIV table (Format / Headers / Content = Yes; MT300 &amp; FX S reports matched 11/14 versus 11/15)</t>
         </is>
       </c>
@@ -21967,7 +21975,7 @@
       </c>
       <c r="J9" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 61, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 61, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 62, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, BCiC report screen (record on a later page of the 66-item report)
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 25
@@ -21988,7 +21996,7 @@
           <t>E05: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg, IT DR: 2025 BIA results &amp; applications list review (invite 09/15/2025, re-sent 09/18/2025)
 DMA02: BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg, attached signed attestation section 1-2, IT DR team facilitates DIV performed by business line testers during actual DR testing
 BLA04: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx, IT DR test script completed by the business-line tester
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 61, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 61, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M9" s="25" t="inlineStr">
@@ -22071,8 +22079,8 @@
       </c>
       <c r="E10" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 25, 29, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 25, 29 to 11/15/2025; Y / Y / Y
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 25, 29, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 25, 29 to 11/15/2025; Format, Headers and Content validated
 BLA03: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf, pp.1-2 DIV section (Format / Headers / Content = yes; 11/14 Fed &amp; SWIFT data reconciled)
 E07: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg, pre-DR source reports 11/14/2025 (Payment Monitor, OFAC, SWIFT Interface Monitor)
 E08: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg, DR test-day 11/15/2025 comparison reports</t>
@@ -22104,7 +22112,7 @@
       </c>
       <c r="J10" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 25, 29, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 25, 29, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 25, 29, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, BCiC report screen (record on a later page of the 66-item report)
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 31
@@ -22126,7 +22134,7 @@
 DMA02: BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg, attached signed attestation section 1-2, IT DR team facilitates DIV performed by business line testers during actual DR testing
 BLA03: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 E08: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg, business-line DIV comparison files sent to IT DR (Elizabeth Noda) on 11/15/2025
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 25, 29, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 25, 29, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M10" s="25" t="inlineStr">
@@ -22214,9 +22222,9 @@
       </c>
       <c r="E11" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 6, 26, 30, 34, 58, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 6, 26, 30, 34, 59 to 11/15/2025; Y / Y / Y
-E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and Y/N columns
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 6, 26, 30, 34, 58, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 6, 26, 30, 34, 59 to 11/15/2025; Format, Headers and Content validated
+E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and validation result columns
 BLA02: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf, p.1 DIV procedure &amp; in-scope apps; pp.2-14 production-day 11/14 versus test-day 11/15 screenshots
 BLA03: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf, pp.1-2 DIV section (Format / Headers / Content = yes; 11/14 Fed &amp; SWIFT data reconciled)
 E07: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg, pre-DR source reports 11/14/2025 (Payment Monitor, OFAC, SWIFT Interface Monitor)
@@ -22258,7 +22266,7 @@
       </c>
       <c r="J11" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 6, 26, 30, 34, 58, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 6, 26, 30, 34, 58, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 6, 26, 30, 34, 59, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, records visible on screen
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 34
@@ -22282,7 +22290,7 @@
 BLA02: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 BLA03: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 E08: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg, business-line DIV comparison files sent to IT DR (Elizabeth Noda) on 11/15/2025
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 6, 26, 30, 34, 58, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 6, 26, 30, 34, 58, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M11" s="25" t="inlineStr">
@@ -22372,8 +22380,8 @@
       </c>
       <c r="E12" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 17, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 17 to 11/15/2025; Y / Y / Y
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 17, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 17 to 11/15/2025; Format, Headers and Content validated
 BLA05: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Yes / Yes / Yes, no discrepancies); pp.2-9 reconciliation reports 11/13 versus 11/15</t>
         </is>
       </c>
@@ -22403,7 +22411,7 @@
       </c>
       <c r="J12" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 17, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 17, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, row 17, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, BCiC report screen (record on a later page of the 66-item report)
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 36
@@ -22425,7 +22433,7 @@
 DMA02: BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg, attached signed attestation section 1-2, IT DR team facilitates DIV performed by business line testers during actual DR testing
 BLA05: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 E10: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg, IT DR (Elizabeth Noda) Finance DIV chart and approval request
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 17, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, row 17, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M12" s="25" t="inlineStr">
@@ -22512,9 +22520,9 @@
       </c>
       <c r="E13" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 7, 60, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 7, 61 to 11/15/2025; Y / Y / Y
-E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and Y/N columns
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 7, 60, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 7, 61 to 11/15/2025; Format, Headers and Content validated
+E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and validation result columns
 BLA03: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf, pp.1-2 DIV section (Format / Headers / Content = yes; 11/14 Fed &amp; SWIFT data reconciled)
 BLA04: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx, DIV table (Format / Headers / Content = Yes; MT300 &amp; FX S reports matched 11/14 versus 11/15)
 E07: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg, pre-DR source reports 11/14/2025 (Payment Monitor, OFAC, SWIFT Interface Monitor)
@@ -22553,7 +22561,7 @@
       </c>
       <c r="J13" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 7, 60, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 7, 60, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 7, 61, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, records visible on screen
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 42
@@ -22577,7 +22585,7 @@
 BLA03: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 BLA04: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx, IT DR test script completed by the business-line tester
 E08: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg, business-line DIV comparison files sent to IT DR (Elizabeth Noda) on 11/15/2025
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 7, 60, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 7, 60, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M13" s="25" t="inlineStr">
@@ -22674,10 +22682,10 @@
       </c>
       <c r="E14" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 3, 8, 12, 14, 15, 16, 18, 19, 20, 21, 23, 27, 31, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 48, 49, 50, 52, 54, 55, 56, 59, 62, 63, Business Data Validation Date 11/15/2025; Y/N Format / Headers / Content = Y
-E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 3, 8, 12, 14, 15, 16, 18, 19, 20, 21, 23, 27, 31, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 49, 50, 51, 53, 55, 56, 57, 60, 63, 64 to 11/15/2025; Y / Y / Y
-E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and Y/N columns
-BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format / Headers / Content = Y, "No data discrepancy found"); pp.2-14 screenshots
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 3, 8, 12, 14, 15, 16, 18, 19, 20, 21, 23, 27, 31, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 48, 49, 50, 52, 54, 55, 56, 59, 62, 63, Business Data Validation Date 11/15/2025; Format, Headers and Content validated
+E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 3, 8, 12, 14, 15, 16, 18, 19, 20, 21, 23, 27, 31, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 49, 50, 51, 53, 55, 56, 57, 60, 63, 64 to 11/15/2025; Format, Headers and Content validated
+E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, Business Data Validation Date and validation result columns
+BLA01: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf, p.1 DIV section (Format, Headers and Content validated, "No data discrepancy found"); pp.2-14 screenshots
 BLA02: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf, p.1 DIV procedure &amp; in-scope apps; pp.2-14 production-day 11/14 versus test-day 11/15 screenshots
 BLA03: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf, pp.1-2 DIV section (Format / Headers / Content = yes; 11/14 Fed &amp; SWIFT data reconciled)
 BLA04: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx, DIV table (Format / Headers / Content = Yes; MT300 &amp; FX S reports matched 11/14 versus 11/15)
@@ -22757,7 +22765,7 @@
       </c>
       <c r="J14" s="25" t="inlineStr">
         <is>
-          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 3, 8, 12, 14, 15, 16, 18, 19, 20, 21, 23, 27, 31, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 48, 49, 50, 52, 54, 55, 56, 59, 62, 63, BCiC DIV export (tester, dates, manager, Y/N results, attestation)
+          <t>E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 3, 8, 12, 14, 15, 16, 18, 19, 20, 21, 23, 27, 31, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 48, 49, 50, 52, 54, 55, 56, 59, 62, 63, BCiC DIV export (tester, dates, manager, validation results, attestation)
 E16b: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx, rows 3, 8, 12, 14, 15, 16, 18, 19, 20, 21, 23, 27, 31, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 49, 50, 51, 53, 55, 56, 57, 60, 63, 64, BCiC DIV export 2025-26 reviewed with the attestation
 E04: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg, records visible on screen
 E01: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx, row 43
@@ -22788,7 +22796,7 @@
 BLA05: BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf, IT DR test script completed by the business-line tester
 E08: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg, business-line DIV comparison files sent to IT DR (Elizabeth Noda) on 11/15/2025
 E10: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg, IT DR (Elizabeth Noda) Finance DIV chart and approval request
-E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 3, 8, 12, 14, 15, 16, 18, 19, 20, 21, 23, 27, 31, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 48, 49, 50, 52, 54, 55, 56, 59, 62, 63, Y/N Format, Headers, Content = Y</t>
+E03: BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls, rows 3, 8, 12, 14, 15, 16, 18, 19, 20, 21, 23, 27, 31, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 48, 49, 50, 52, 54, 55, 56, 59, 62, 63, Format, Headers and Content validated</t>
         </is>
       </c>
       <c r="M14" s="25" t="inlineStr">
@@ -23142,7 +23150,7 @@
       </c>
       <c r="H4" s="35" t="inlineStr">
         <is>
-          <t>DR test script with Data Integrity Validation section. Application in-scope: FedImport, FedExport, Imaging101, T24. Format / Headers / Content = Y, "No data discrepancy found". Steps include ACH Express import and Imaging101 validation screenshots (14 pages).</t>
+          <t>DR test script with Data Integrity Validation section. Application in-scope: FedImport, FedExport, Imaging101, T24. Format, Headers and Content validated, "No data discrepancy found". Steps include ACH Express import and Imaging101 validation screenshots (14 pages).</t>
         </is>
       </c>
       <c r="I4" s="35" t="inlineStr">
@@ -23506,7 +23514,7 @@
       </c>
       <c r="H11" s="35" t="inlineStr">
         <is>
-          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all Y/Y/Y; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.</t>
+          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf, signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation section 1: IT DR team facilitates DIV annually; section 2: 63 entries / 13 applications, all validated; section 3.5: retained in BCMS/BCiC; section 3.6: contemporaneous approval going forward.</t>
         </is>
       </c>
       <c r="I11" s="35" t="inlineStr">
@@ -24230,7 +24238,7 @@
       </c>
       <c r="H25" s="35" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Format/Headers/Content validation results, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
         </is>
       </c>
       <c r="I25" s="35" t="inlineStr">
@@ -24282,7 +24290,7 @@
       </c>
       <c r="H26" s="35" t="inlineStr">
         <is>
-          <t>BCiC 'Data Integrity Validation Testing' screen (1 to 20 of 66 items) showing tester, validation date, manager, approval date, Y/N results and attestation fields.</t>
+          <t>BCiC 'Data Integrity Validation Testing' screen (1 to 20 of 66 items) showing tester, validation date, manager, approval date, validation results and attestation fields.</t>
         </is>
       </c>
       <c r="I26" s="35" t="inlineStr">

</xml_diff>

<commit_message>
Workpaper 13_1: add annual-execution note to tab -2 attribute 12
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TL6bHHvGD5mcHDaTAY6zMH
</commit_message>
<xml_diff>
--- a/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_13_1.xlsx
+++ b/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_13_1.xlsx
@@ -1386,6 +1386,11 @@
         <t>Annual execution: 2025 cycle, BSI IT DR Exercise 11/15/2025 (DIV validated 11/15/2025), within the review period 08/01/2025 to 06/01/2026. 2024 cycle, Full DR Test (Virginia) 10/19/2024, see tab 'DR 2024 Testing Results'. One DR / DIV exercise per annual cycle; 392 days between exercises.</t>
       </text>
     </comment>
+    <comment ref="A51" authorId="1" shapeId="0">
+      <text>
+        <t>Yes, annually executed. 2025 cycle: BSI IT DR Exercise 11/15/2025 (DIV validated 11/15/2025), within the review period 08/01/2025 to 06/01/2026. 2024 cycle: 2024 Full 2024 DR Test (Virginia) on 10/19/2024, see tab 'DR 2024 Testing Results' (application not listed individually on that extract). One DR / DIV exercise executed in each annual DR cycle; interval 10/19/2024 to 11/15/2025 = 392 days.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -13970,7 +13975,7 @@
       <c r="AX52" s="85" t="n"/>
       <c r="AY52" s="85" t="n"/>
     </row>
-    <row r="53" ht="126" customHeight="1" s="50">
+    <row r="53" ht="200" customHeight="1" s="50">
       <c r="A53" s="78" t="inlineStr">
         <is>
           <t>E01</t>
@@ -14004,7 +14009,8 @@
           <t>BCiC export of the BSI DR-scope population (43 applications) with Exercise Date and 2025 DR / Backup-Restore / DIV scope flags.
 Checked for Annual Testing Executed:
 Exercise Date 12/11/2025 / 2025 DR Test Scope = True
-Exercise Date 11/15/2025 / 2025 DR Test Scope = True</t>
+Exercise Date 11/15/2025 / 2025 DR Test Scope = True
+Note: Yes, annually executed. 2025 cycle: BSI IT DR Exercise 11/15/2025 (DIV validated 11/15/2025), within the review period 08/01/2025 to 06/01/2026. 2024 cycle: 2024 Full 2024 DR Test (Virginia) on 10/19/2024, see tab 'DR 2024 Testing Results' (application not listed individually on that extract). One DR / DIV exercise executed in each annual DR cycle; interval 10/19/2024 to 11/15/2025 = 392 days.</t>
         </is>
       </c>
       <c r="F53" s="76" t="inlineStr">

</xml_diff>